<commit_message>
Automatsko ažuriranje artikli.xlsx iz POS sistema
</commit_message>
<xml_diff>
--- a/artikli.xlsx
+++ b/artikli.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4867"/>
+  <dimension ref="A1:D4929"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>ELLA GEL ZA KOSU</t>
+          <t>ELLA GEL ZA KOSU PLAVI 250ML</t>
         </is>
       </c>
       <c r="D149" t="n">
@@ -6951,7 +6951,7 @@
         </is>
       </c>
       <c r="D363" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="364">
@@ -8265,7 +8265,7 @@
         </is>
       </c>
       <c r="D436" t="n">
-        <v>26</v>
+        <v>27.5</v>
       </c>
     </row>
     <row r="437">
@@ -8801,7 +8801,7 @@
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>STARK KAKAO KEKSICI 220 G</t>
+          <t>STARK KAKAO KEKSICI 220G</t>
         </is>
       </c>
       <c r="D466" t="n">
@@ -8963,7 +8963,7 @@
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>BAJADERA 300 G</t>
+          <t>BAJADERA 300G</t>
         </is>
       </c>
       <c r="D475" t="n">
@@ -11429,7 +11429,7 @@
       </c>
       <c r="C612" t="inlineStr">
         <is>
-          <t>KIKI 100 G</t>
+          <t>KIKI 100G</t>
         </is>
       </c>
       <c r="D612" t="n">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="C615" t="inlineStr">
         <is>
-          <t>BELA MENTA 100 G</t>
+          <t>BELA MENTA 100G</t>
         </is>
       </c>
       <c r="D615" t="n">
@@ -12635,7 +12635,7 @@
       </c>
       <c r="C679" t="inlineStr">
         <is>
-          <t>SMOKI 40 G</t>
+          <t>SMOKI STARK 40G</t>
         </is>
       </c>
       <c r="D679" t="n">
@@ -13013,7 +13013,7 @@
       </c>
       <c r="C700" t="inlineStr">
         <is>
-          <t>SMOKI STARK 130 G</t>
+          <t>SMOKI STARK 130G</t>
         </is>
       </c>
       <c r="D700" t="n">
@@ -15803,7 +15803,7 @@
       </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>DESERTNI PRELJEV OD COKOLADE 350 G</t>
+          <t>DESERTNI PRELIV OD COKOLADE 350G</t>
         </is>
       </c>
       <c r="D855" t="n">
@@ -16275,7 +16275,7 @@
         </is>
       </c>
       <c r="D881" t="n">
-        <v>5.8</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="882">
@@ -21603,7 +21603,7 @@
         </is>
       </c>
       <c r="D1177" t="n">
-        <v>2.1</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="1178">
@@ -22049,7 +22049,7 @@
       </c>
       <c r="C1202" t="inlineStr">
         <is>
-          <t>ALU FOLIJA 1 KG</t>
+          <t>FRESH ALU FOLIJA  290MM 1KG</t>
         </is>
       </c>
       <c r="D1202" t="n">
@@ -24407,7 +24407,7 @@
       </c>
       <c r="C1333" t="inlineStr">
         <is>
-          <t>BRONHI BOMBONE 100 G</t>
+          <t>BRONHI BOMBONE 100G</t>
         </is>
       </c>
       <c r="D1333" t="n">
@@ -24659,11 +24659,11 @@
       </c>
       <c r="C1347" t="inlineStr">
         <is>
-          <t>MEKSIKANA SALATA SA TUNJEVINOM TREND 160 G</t>
+          <t>TREND MEKS. SALATA SA TUNJ. 160G</t>
         </is>
       </c>
       <c r="D1347" t="n">
-        <v>3.5</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="1348">
@@ -25253,11 +25253,11 @@
       </c>
       <c r="C1380" t="inlineStr">
         <is>
-          <t>SLAG U SPREJU</t>
+          <t>MONTARE SLAG U SPREJU 250G</t>
         </is>
       </c>
       <c r="D1380" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="1381">
@@ -30113,7 +30113,7 @@
       </c>
       <c r="C1650" t="inlineStr">
         <is>
-          <t>COCA-COLA ZERO 0,5 L</t>
+          <t>COCA-COLA ZERO 0,5L</t>
         </is>
       </c>
       <c r="D1650" t="n">
@@ -30347,7 +30347,7 @@
       </c>
       <c r="C1663" t="inlineStr">
         <is>
-          <t>VODA PROLOM 0,5 L</t>
+          <t>VODA PROLOM 0,5L</t>
         </is>
       </c>
       <c r="D1663" t="n">
@@ -30743,7 +30743,7 @@
       </c>
       <c r="C1685" t="inlineStr">
         <is>
-          <t>JANA VITAMIN LIMUN IMUNO 0,5 L</t>
+          <t>JANA VITAMIN LIMUN IMUNO 0,5L</t>
         </is>
       </c>
       <c r="D1685" t="n">
@@ -31157,7 +31157,7 @@
       </c>
       <c r="C1708" t="inlineStr">
         <is>
-          <t>JUICY FRUITS MULTIVITAMIN 2 L</t>
+          <t>JUICY FRUITS MULTIVITAMIN 2L</t>
         </is>
       </c>
       <c r="D1708" t="n">
@@ -33591,7 +33591,7 @@
         </is>
       </c>
       <c r="D1843" t="n">
-        <v>4.8</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="1844">
@@ -35603,11 +35603,11 @@
       </c>
       <c r="C1955" t="inlineStr">
         <is>
-          <t>POSUDA 1,7 L</t>
+          <t>POSUDA 1,7L DRINA</t>
         </is>
       </c>
       <c r="D1955" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="1956">
@@ -40665,7 +40665,7 @@
         </is>
       </c>
       <c r="D2236" t="n">
-        <v>12.5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2237">
@@ -43901,7 +43901,7 @@
       </c>
       <c r="C2416" t="inlineStr">
         <is>
-          <t>FRUTEK JABUKA</t>
+          <t>FRUTEK JABUKA 125ML</t>
         </is>
       </c>
       <c r="D2416" t="n">
@@ -44639,7 +44639,7 @@
       </c>
       <c r="C2457" t="inlineStr">
         <is>
-          <t>GRIL PREMIUM BRIKETI 2,50</t>
+          <t>GRIL PREMIUM BRIKETI 2,50KG</t>
         </is>
       </c>
       <c r="D2457" t="n">
@@ -47375,7 +47375,7 @@
       </c>
       <c r="C2609" t="inlineStr">
         <is>
-          <t>ELLA GEL ZA KOSU</t>
+          <t>ELLA GEL ZA KOSU BIJELI 250ML</t>
         </is>
       </c>
       <c r="D2609" t="n">
@@ -50799,7 +50799,7 @@
         </is>
       </c>
       <c r="D2799" t="n">
-        <v>2.3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="2800">
@@ -58341,7 +58341,7 @@
         </is>
       </c>
       <c r="D3218" t="n">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="3219">
@@ -58413,7 +58413,7 @@
         </is>
       </c>
       <c r="D3222" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="3223">
@@ -59705,11 +59705,11 @@
       </c>
       <c r="C3294" t="inlineStr">
         <is>
-          <t>POSUDA 2,5L</t>
+          <t>POSUDA 2,5L DRINA</t>
         </is>
       </c>
       <c r="D3294" t="n">
-        <v>3.7</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="3295">
@@ -82767,7 +82767,7 @@
         </is>
       </c>
       <c r="D4575" t="n">
-        <v>6.9</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="4576">
@@ -87659,7 +87659,7 @@
       </c>
       <c r="C4847" t="inlineStr">
         <is>
-          <t>MIRISNA SPUZVA 2,/4 NARANDZA</t>
+          <t>MIRISNA SPUZVA 2/4 NARANDZA</t>
         </is>
       </c>
       <c r="D4847" t="n">
@@ -88024,6 +88024,1122 @@
       </c>
       <c r="D4867" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="4868">
+      <c r="A4868" t="n">
+        <v>4867</v>
+      </c>
+      <c r="B4868" t="inlineStr">
+        <is>
+          <t>3838945004042</t>
+        </is>
+      </c>
+      <c r="C4868" t="inlineStr">
+        <is>
+          <t>DVOJNI C INSTANT LIMUN 200G</t>
+        </is>
+      </c>
+      <c r="D4868" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="4869">
+      <c r="A4869" t="n">
+        <v>4868</v>
+      </c>
+      <c r="B4869" t="inlineStr">
+        <is>
+          <t>3838945044035</t>
+        </is>
+      </c>
+      <c r="C4869" t="inlineStr">
+        <is>
+          <t>DVOJNI C INSTANT NARANDZA 500G</t>
+        </is>
+      </c>
+      <c r="D4869" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="4870">
+      <c r="A4870" t="n">
+        <v>4869</v>
+      </c>
+      <c r="B4870" t="inlineStr">
+        <is>
+          <t>3871862002696</t>
+        </is>
+      </c>
+      <c r="C4870" t="inlineStr">
+        <is>
+          <t>TREND DJUVEC 850G</t>
+        </is>
+      </c>
+      <c r="D4870" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="4871">
+      <c r="A4871" t="n">
+        <v>4870</v>
+      </c>
+      <c r="B4871" t="inlineStr">
+        <is>
+          <t>8714800011426</t>
+        </is>
+      </c>
+      <c r="C4871" t="inlineStr">
+        <is>
+          <t>BAVARIA 0.5L BEZALKOHOLO PIVO</t>
+        </is>
+      </c>
+      <c r="D4871" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="4872">
+      <c r="A4872" t="n">
+        <v>4871</v>
+      </c>
+      <c r="B4872" t="inlineStr">
+        <is>
+          <t>3870343000619</t>
+        </is>
+      </c>
+      <c r="C4872" t="inlineStr">
+        <is>
+          <t>SOCIVICA 800G MALPAK</t>
+        </is>
+      </c>
+      <c r="D4872" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="4873">
+      <c r="A4873" t="n">
+        <v>4872</v>
+      </c>
+      <c r="B4873" t="inlineStr">
+        <is>
+          <t>8032793344308</t>
+        </is>
+      </c>
+      <c r="C4873" t="inlineStr">
+        <is>
+          <t>POMI PASIRANA RAJCICA 200G</t>
+        </is>
+      </c>
+      <c r="D4873" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="4874">
+      <c r="A4874" t="n">
+        <v>4873</v>
+      </c>
+      <c r="B4874" t="inlineStr">
+        <is>
+          <t>8606012145122</t>
+        </is>
+      </c>
+      <c r="C4874" t="inlineStr">
+        <is>
+          <t>KOSILI SP.P.UB.KOM. I KRP. 100ML</t>
+        </is>
+      </c>
+      <c r="D4874" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4875">
+      <c r="A4875" t="n">
+        <v>4874</v>
+      </c>
+      <c r="B4875" t="inlineStr">
+        <is>
+          <t>8606012145092</t>
+        </is>
+      </c>
+      <c r="C4875" t="inlineStr">
+        <is>
+          <t>LMX SP. PR. KOM. I KRPELJA 100ML</t>
+        </is>
+      </c>
+      <c r="D4875" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="4876">
+      <c r="A4876" t="n">
+        <v>4875</v>
+      </c>
+      <c r="B4876" t="inlineStr">
+        <is>
+          <t>8007150901951</t>
+        </is>
+      </c>
+      <c r="C4876" t="inlineStr">
+        <is>
+          <t>OLITALIA ACETO BALSAMICO 500ML</t>
+        </is>
+      </c>
+      <c r="D4876" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="4877">
+      <c r="A4877" t="n">
+        <v>4876</v>
+      </c>
+      <c r="B4877" t="inlineStr">
+        <is>
+          <t>3870254000845</t>
+        </is>
+      </c>
+      <c r="C4877" t="inlineStr">
+        <is>
+          <t>SALBOS SO ZA MASINU LIMUN 1.5KG</t>
+        </is>
+      </c>
+      <c r="D4877" t="n">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="4878">
+      <c r="A4878" t="n">
+        <v>4877</v>
+      </c>
+      <c r="B4878" t="inlineStr">
+        <is>
+          <t>3870254000593</t>
+        </is>
+      </c>
+      <c r="C4878" t="inlineStr">
+        <is>
+          <t>SALBON SO ZA MASINU 1.5KG</t>
+        </is>
+      </c>
+      <c r="D4878" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="4879">
+      <c r="A4879" t="n">
+        <v>4878</v>
+      </c>
+      <c r="B4879" t="inlineStr">
+        <is>
+          <t>3870022005188</t>
+        </is>
+      </c>
+      <c r="C4879" t="inlineStr">
+        <is>
+          <t>DITA DESTILOVANA VODA 1L</t>
+        </is>
+      </c>
+      <c r="D4879" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="4880">
+      <c r="A4880" t="n">
+        <v>4879</v>
+      </c>
+      <c r="B4880" t="inlineStr">
+        <is>
+          <t>3870022005065</t>
+        </is>
+      </c>
+      <c r="C4880" t="inlineStr">
+        <is>
+          <t>DITA DESTILOVANA VODA 5L</t>
+        </is>
+      </c>
+      <c r="D4880" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="4881">
+      <c r="A4881" t="n">
+        <v>4880</v>
+      </c>
+      <c r="B4881" t="inlineStr">
+        <is>
+          <t>8606112009515</t>
+        </is>
+      </c>
+      <c r="C4881" t="inlineStr">
+        <is>
+          <t>EP PAPIR ZA PECENJE 16/1 42X38</t>
+        </is>
+      </c>
+      <c r="D4881" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4882">
+      <c r="A4882" t="n">
+        <v>4881</v>
+      </c>
+      <c r="B4882" t="inlineStr">
+        <is>
+          <t>8605062104554</t>
+        </is>
+      </c>
+      <c r="C4882" t="inlineStr">
+        <is>
+          <t>VODENI PISTOLJ DELFIN</t>
+        </is>
+      </c>
+      <c r="D4882" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4883">
+      <c r="A4883" t="n">
+        <v>4882</v>
+      </c>
+      <c r="B4883" t="inlineStr">
+        <is>
+          <t>3850104295096</t>
+        </is>
+      </c>
+      <c r="C4883" t="inlineStr">
+        <is>
+          <t>FANT TJEST. SA 4 VRSTE SIRA 53G</t>
+        </is>
+      </c>
+      <c r="D4883" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="4884">
+      <c r="A4884" t="n">
+        <v>4883</v>
+      </c>
+      <c r="B4884" t="inlineStr">
+        <is>
+          <t>3838945040815</t>
+        </is>
+      </c>
+      <c r="C4884" t="inlineStr">
+        <is>
+          <t>DVOJNI C 0.25L LIMENKA</t>
+        </is>
+      </c>
+      <c r="D4884" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4885">
+      <c r="A4885" t="n">
+        <v>4884</v>
+      </c>
+      <c r="B4885" t="inlineStr">
+        <is>
+          <t>3838945503013</t>
+        </is>
+      </c>
+      <c r="C4885" t="inlineStr">
+        <is>
+          <t>FRTUEK KASICA 120G JABUKA</t>
+        </is>
+      </c>
+      <c r="D4885" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="4886">
+      <c r="A4886" t="n">
+        <v>4885</v>
+      </c>
+      <c r="B4886" t="inlineStr">
+        <is>
+          <t>5999563941248</t>
+        </is>
+      </c>
+      <c r="C4886" t="inlineStr">
+        <is>
+          <t>KING HRANA ZA PSE PILETINA 1240G</t>
+        </is>
+      </c>
+      <c r="D4886" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4887">
+      <c r="A4887" t="n">
+        <v>4886</v>
+      </c>
+      <c r="B4887" t="inlineStr">
+        <is>
+          <t>3856016327284</t>
+        </is>
+      </c>
+      <c r="C4887" t="inlineStr">
+        <is>
+          <t>MARGO NOVA MARG. 225G</t>
+        </is>
+      </c>
+      <c r="D4887" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4888">
+      <c r="A4888" t="n">
+        <v>4887</v>
+      </c>
+      <c r="B4888" t="inlineStr">
+        <is>
+          <t>3838945521161</t>
+        </is>
+      </c>
+      <c r="C4888" t="inlineStr">
+        <is>
+          <t>FRUCTAL NATURA CVEKLA 100% 700ML</t>
+        </is>
+      </c>
+      <c r="D4888" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4889">
+      <c r="A4889" t="n">
+        <v>4888</v>
+      </c>
+      <c r="B4889" t="inlineStr">
+        <is>
+          <t>3838945044028</t>
+        </is>
+      </c>
+      <c r="C4889" t="inlineStr">
+        <is>
+          <t>DVOJNI C INSTANT NARANDZA 200G</t>
+        </is>
+      </c>
+      <c r="D4889" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4890">
+      <c r="A4890" t="n">
+        <v>4889</v>
+      </c>
+      <c r="B4890" t="inlineStr">
+        <is>
+          <t>8600169500022</t>
+        </is>
+      </c>
+      <c r="C4890" t="inlineStr">
+        <is>
+          <t>PROLOM VODA 1.5</t>
+        </is>
+      </c>
+      <c r="D4890" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4891">
+      <c r="A4891" t="n">
+        <v>4890</v>
+      </c>
+      <c r="B4891" t="inlineStr">
+        <is>
+          <t>3872216000008</t>
+        </is>
+      </c>
+      <c r="C4891" t="inlineStr">
+        <is>
+          <t>ARGETA KOKOSIJA PASTETA 95G</t>
+        </is>
+      </c>
+      <c r="D4891" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4892">
+      <c r="A4892" t="n">
+        <v>4891</v>
+      </c>
+      <c r="B4892" t="inlineStr">
+        <is>
+          <t>3600114011248</t>
+        </is>
+      </c>
+      <c r="C4892" t="inlineStr">
+        <is>
+          <t>JAFFA NAPOL. COKO&amp;NAR. 160G</t>
+        </is>
+      </c>
+      <c r="D4892" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4893">
+      <c r="A4893" t="n">
+        <v>4892</v>
+      </c>
+      <c r="B4893" t="inlineStr">
+        <is>
+          <t>185988858336</t>
+        </is>
+      </c>
+      <c r="C4893" t="inlineStr">
+        <is>
+          <t>ABC SIRNI NAMAZ 200G</t>
+        </is>
+      </c>
+      <c r="D4893" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4894">
+      <c r="A4894" t="n">
+        <v>4893</v>
+      </c>
+      <c r="B4894" t="inlineStr">
+        <is>
+          <t>3858890674044</t>
+        </is>
+      </c>
+      <c r="C4894" t="inlineStr">
+        <is>
+          <t>JANA VITAM. HAPPY NARANDZA 1,5L</t>
+        </is>
+      </c>
+      <c r="D4894" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="4895">
+      <c r="A4895" t="n">
+        <v>4894</v>
+      </c>
+      <c r="B4895" t="inlineStr">
+        <is>
+          <t>8500169600022</t>
+        </is>
+      </c>
+      <c r="C4895" t="inlineStr">
+        <is>
+          <t>PROLOM VODA 1,5L</t>
+        </is>
+      </c>
+      <c r="D4895" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4896">
+      <c r="A4896" t="n">
+        <v>4895</v>
+      </c>
+      <c r="B4896" t="inlineStr">
+        <is>
+          <t>4250443474654</t>
+        </is>
+      </c>
+      <c r="C4896" t="inlineStr">
+        <is>
+          <t>HOLZKOHLE DRVENI UGALJ 2,25KG</t>
+        </is>
+      </c>
+      <c r="D4896" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="4897">
+      <c r="A4897" t="n">
+        <v>4896</v>
+      </c>
+      <c r="B4897" t="inlineStr">
+        <is>
+          <t>4250443474661</t>
+        </is>
+      </c>
+      <c r="C4897" t="inlineStr">
+        <is>
+          <t>HOLZKOHLE DRVENI UGALJ 2,25KG</t>
+        </is>
+      </c>
+      <c r="D4897" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="4898">
+      <c r="A4898" t="n">
+        <v>4897</v>
+      </c>
+      <c r="B4898" t="inlineStr">
+        <is>
+          <t>3871862004706</t>
+        </is>
+      </c>
+      <c r="C4898" t="inlineStr">
+        <is>
+          <t>LUMAX DRVENI UGALJ 2KG</t>
+        </is>
+      </c>
+      <c r="D4898" t="n">
+        <v>6.3</v>
+      </c>
+    </row>
+    <row r="4899">
+      <c r="A4899" t="n">
+        <v>4898</v>
+      </c>
+      <c r="B4899" t="inlineStr">
+        <is>
+          <t>3859888141179</t>
+        </is>
+      </c>
+      <c r="C4899" t="inlineStr">
+        <is>
+          <t>MR. FIRE GRILL BRIKTER 2,5KG</t>
+        </is>
+      </c>
+      <c r="D4899" t="n">
+        <v>7.9</v>
+      </c>
+    </row>
+    <row r="4900">
+      <c r="A4900" t="n">
+        <v>4899</v>
+      </c>
+      <c r="B4900" t="inlineStr">
+        <is>
+          <t>8600104004540</t>
+        </is>
+      </c>
+      <c r="C4900" t="inlineStr">
+        <is>
+          <t>STRUDLE KAJSIJA 240G</t>
+        </is>
+      </c>
+      <c r="D4900" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4901">
+      <c r="A4901" t="n">
+        <v>4900</v>
+      </c>
+      <c r="B4901" t="inlineStr">
+        <is>
+          <t>8600104004632</t>
+        </is>
+      </c>
+      <c r="C4901" t="inlineStr">
+        <is>
+          <t>STRUDLE VISNJA 2,40G</t>
+        </is>
+      </c>
+      <c r="D4901" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4902">
+      <c r="A4902" t="n">
+        <v>4901</v>
+      </c>
+      <c r="B4902" t="inlineStr">
+        <is>
+          <t>600104004748</t>
+        </is>
+      </c>
+      <c r="C4902" t="inlineStr">
+        <is>
+          <t>STRUDLE MIJESANA 360G</t>
+        </is>
+      </c>
+      <c r="D4902" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="4903">
+      <c r="A4903" t="n">
+        <v>4902</v>
+      </c>
+      <c r="B4903" t="inlineStr">
+        <is>
+          <t>8600046004844</t>
+        </is>
+      </c>
+      <c r="C4903" t="inlineStr">
+        <is>
+          <t>BONZITA MALINA JOGURT 28G</t>
+        </is>
+      </c>
+      <c r="D4903" t="n">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4904">
+      <c r="A4904" t="n">
+        <v>4903</v>
+      </c>
+      <c r="B4904" t="inlineStr">
+        <is>
+          <t>3870398907208</t>
+        </is>
+      </c>
+      <c r="C4904" t="inlineStr">
+        <is>
+          <t>CVJETACA 400G</t>
+        </is>
+      </c>
+      <c r="D4904" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="4905">
+      <c r="A4905" t="n">
+        <v>4904</v>
+      </c>
+      <c r="B4905" t="inlineStr">
+        <is>
+          <t>5948351012875</t>
+        </is>
+      </c>
+      <c r="C4905" t="inlineStr">
+        <is>
+          <t>POK. VREC RIBE PLAVA</t>
+        </is>
+      </c>
+      <c r="D4905" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="4906">
+      <c r="A4906" t="n">
+        <v>4905</v>
+      </c>
+      <c r="B4906" t="inlineStr">
+        <is>
+          <t>5900928007264</t>
+        </is>
+      </c>
+      <c r="C4906" t="inlineStr">
+        <is>
+          <t>DIJO GRILLED TORTILJA 250G</t>
+        </is>
+      </c>
+      <c r="D4906" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="4907">
+      <c r="A4907" t="n">
+        <v>4906</v>
+      </c>
+      <c r="B4907" t="inlineStr">
+        <is>
+          <t>8610056050212</t>
+        </is>
+      </c>
+      <c r="C4907" t="inlineStr">
+        <is>
+          <t>SET KERAMICKIH ZDJELICA 4/1</t>
+        </is>
+      </c>
+      <c r="D4907" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="4908">
+      <c r="A4908" t="n">
+        <v>4907</v>
+      </c>
+      <c r="B4908" t="inlineStr">
+        <is>
+          <t>8610056049476</t>
+        </is>
+      </c>
+      <c r="C4908" t="inlineStr">
+        <is>
+          <t>SET KER. ZDJ. SA KASICICAMA 4/1</t>
+        </is>
+      </c>
+      <c r="D4908" t="n">
+        <v>13.2</v>
+      </c>
+    </row>
+    <row r="4909">
+      <c r="A4909" t="n">
+        <v>4908</v>
+      </c>
+      <c r="B4909" t="inlineStr">
+        <is>
+          <t>8610056049544</t>
+        </is>
+      </c>
+      <c r="C4909" t="inlineStr">
+        <is>
+          <t>SET KER. OVALA 2/1</t>
+        </is>
+      </c>
+      <c r="D4909" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4910">
+      <c r="A4910" t="n">
+        <v>4909</v>
+      </c>
+      <c r="B4910" t="inlineStr">
+        <is>
+          <t>7988896535895</t>
+        </is>
+      </c>
+      <c r="C4910" t="inlineStr">
+        <is>
+          <t>TAVA ZA PALACINKE 24CM</t>
+        </is>
+      </c>
+      <c r="D4910" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4911">
+      <c r="A4911" t="n">
+        <v>4910</v>
+      </c>
+      <c r="B4911" t="inlineStr">
+        <is>
+          <t>6260361069250</t>
+        </is>
+      </c>
+      <c r="C4911" t="inlineStr">
+        <is>
+          <t>BOKAL MAYA 2000ML</t>
+        </is>
+      </c>
+      <c r="D4911" t="n">
+        <v>8.4</v>
+      </c>
+    </row>
+    <row r="4912">
+      <c r="A4912" t="n">
+        <v>4911</v>
+      </c>
+      <c r="B4912" t="inlineStr">
+        <is>
+          <t>8610056048615</t>
+        </is>
+      </c>
+      <c r="C4912" t="inlineStr">
+        <is>
+          <t>ZDJELA 2500ML 25X9CM</t>
+        </is>
+      </c>
+      <c r="D4912" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4913">
+      <c r="A4913" t="n">
+        <v>4912</v>
+      </c>
+      <c r="B4913" t="inlineStr">
+        <is>
+          <t>8610056048622</t>
+        </is>
+      </c>
+      <c r="C4913" t="inlineStr">
+        <is>
+          <t>ZDJELA 1500ML 20X7,5CM</t>
+        </is>
+      </c>
+      <c r="D4913" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4914">
+      <c r="A4914" t="n">
+        <v>4913</v>
+      </c>
+      <c r="B4914" t="inlineStr">
+        <is>
+          <t>8610056048608</t>
+        </is>
+      </c>
+      <c r="C4914" t="inlineStr">
+        <is>
+          <t>ZDJELA 4400ML 30X10,7CM</t>
+        </is>
+      </c>
+      <c r="D4914" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4915">
+      <c r="A4915" t="n">
+        <v>4914</v>
+      </c>
+      <c r="B4915" t="inlineStr">
+        <is>
+          <t>6943750903624</t>
+        </is>
+      </c>
+      <c r="C4915" t="inlineStr">
+        <is>
+          <t>KOMPOT OD BRESKVE 4X120GR</t>
+        </is>
+      </c>
+      <c r="D4915" t="n">
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="4916">
+      <c r="A4916" t="n">
+        <v>4915</v>
+      </c>
+      <c r="B4916" t="inlineStr">
+        <is>
+          <t>8610056035028</t>
+        </is>
+      </c>
+      <c r="C4916" t="inlineStr">
+        <is>
+          <t>PEKAC 34,5X24X8CM</t>
+        </is>
+      </c>
+      <c r="D4916" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="4917">
+      <c r="A4917" t="n">
+        <v>4916</v>
+      </c>
+      <c r="B4917" t="inlineStr">
+        <is>
+          <t>6924565931255</t>
+        </is>
+      </c>
+      <c r="C4917" t="inlineStr">
+        <is>
+          <t>BRIJAC MUSKI 1/1</t>
+        </is>
+      </c>
+      <c r="D4917" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4918">
+      <c r="A4918" t="n">
+        <v>4917</v>
+      </c>
+      <c r="B4918" t="inlineStr">
+        <is>
+          <t>6924565930340</t>
+        </is>
+      </c>
+      <c r="C4918" t="inlineStr">
+        <is>
+          <t>BRIJAC ZENSKI 1/1</t>
+        </is>
+      </c>
+      <c r="D4918" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4919">
+      <c r="A4919" t="n">
+        <v>4918</v>
+      </c>
+      <c r="B4919" t="inlineStr">
+        <is>
+          <t>5997844301095</t>
+        </is>
+      </c>
+      <c r="C4919" t="inlineStr">
+        <is>
+          <t>PLASTICNA ZICA SA SUDJE 3/1</t>
+        </is>
+      </c>
+      <c r="D4919" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="4920">
+      <c r="A4920" t="n">
+        <v>4919</v>
+      </c>
+      <c r="B4920" t="inlineStr">
+        <is>
+          <t>8696630115546</t>
+        </is>
+      </c>
+      <c r="C4920" t="inlineStr">
+        <is>
+          <t>ALBA COSMETIC SPREJ ZA INS. 400ML</t>
+        </is>
+      </c>
+      <c r="D4920" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="4921">
+      <c r="A4921" t="n">
+        <v>4920</v>
+      </c>
+      <c r="B4921" t="inlineStr">
+        <is>
+          <t>8606003591006</t>
+        </is>
+      </c>
+      <c r="C4921" t="inlineStr">
+        <is>
+          <t>VANGLA 3L DRINA</t>
+        </is>
+      </c>
+      <c r="D4921" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="4922">
+      <c r="A4922" t="n">
+        <v>4921</v>
+      </c>
+      <c r="B4922" t="inlineStr">
+        <is>
+          <t>8606003592256</t>
+        </is>
+      </c>
+      <c r="C4922" t="inlineStr">
+        <is>
+          <t>MIX PUSUDA 5L DRINA</t>
+        </is>
+      </c>
+      <c r="D4922" t="n">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="4923">
+      <c r="A4923" t="n">
+        <v>4922</v>
+      </c>
+      <c r="B4923" t="inlineStr">
+        <is>
+          <t>3850105101075</t>
+        </is>
+      </c>
+      <c r="C4923" t="inlineStr">
+        <is>
+          <t>ARF SRED. ZA CIS. SA PRSKAL. 650ML</t>
+        </is>
+      </c>
+      <c r="D4923" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4924">
+      <c r="A4924" t="n">
+        <v>4923</v>
+      </c>
+      <c r="B4924" t="inlineStr">
+        <is>
+          <t>3850105109545</t>
+        </is>
+      </c>
+      <c r="C4924" t="inlineStr">
+        <is>
+          <t>ARF SRED. ZA CIS. SA PRSKAL. 650ML</t>
+        </is>
+      </c>
+      <c r="D4924" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4925">
+      <c r="A4925" t="n">
+        <v>4924</v>
+      </c>
+      <c r="B4925" t="inlineStr">
+        <is>
+          <t>3875010513476</t>
+        </is>
+      </c>
+      <c r="C4925" t="inlineStr">
+        <is>
+          <t>ARF SRED. ZA CIS. SA PRSKAL. 650ML</t>
+        </is>
+      </c>
+      <c r="D4925" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4926">
+      <c r="A4926" t="n">
+        <v>4925</v>
+      </c>
+      <c r="B4926" t="inlineStr">
+        <is>
+          <t>9000101832990</t>
+        </is>
+      </c>
+      <c r="C4926" t="inlineStr">
+        <is>
+          <t>PERSIL DET. ZA VES PRASK. 9KG</t>
+        </is>
+      </c>
+      <c r="D4926" t="n">
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="4927">
+      <c r="A4927" t="n">
+        <v>4926</v>
+      </c>
+      <c r="B4927" t="inlineStr">
+        <is>
+          <t>3875000031470</t>
+        </is>
+      </c>
+      <c r="C4927" t="inlineStr">
+        <is>
+          <t>EXOTIC ORANGE LIMENKA 0,33L</t>
+        </is>
+      </c>
+      <c r="D4927" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="4928">
+      <c r="A4928" t="n">
+        <v>4927</v>
+      </c>
+      <c r="B4928" t="inlineStr">
+        <is>
+          <t>8445291643796</t>
+        </is>
+      </c>
+      <c r="C4928" t="inlineStr">
+        <is>
+          <t>NES VANILIJA MEGA PACK 14X14G</t>
+        </is>
+      </c>
+      <c r="D4928" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="4929">
+      <c r="A4929" t="n">
+        <v>4928</v>
+      </c>
+      <c r="B4929" t="inlineStr">
+        <is>
+          <t>3870598331851</t>
+        </is>
+      </c>
+      <c r="C4929" t="inlineStr">
+        <is>
+          <t>BLA BLA BLA</t>
+        </is>
+      </c>
+      <c r="D4929" t="n">
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>